<commit_message>
agentic-qe-mvp: release-criteria skill drives Go / Conditional go / No-go; release 2.0 fixes the Flow 1 defects; EQE Flow 2 adds cancellation and gap-story journeys
Co-Authored-By: Devin AI <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/agentic-qe-mvp/demo-artifacts/comparison/compare-CYC-2-vs-CYC-3.xlsx
+++ b/agentic-qe-mvp/demo-artifacts/comparison/compare-CYC-2-vs-CYC-3.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="44">
   <si>
     <t>Artifact</t>
   </si>
@@ -133,25 +133,19 @@
     <t>CYC-3 defects</t>
   </si>
   <si>
-    <t>DEF-007, DEF-008, DEF-010, DEF-011</t>
+    <t>DEF-010</t>
   </si>
   <si>
     <t>new</t>
   </si>
   <si>
-    <t>DEF-010, DEF-011</t>
-  </si>
-  <si>
     <t>still open</t>
   </si>
   <si>
-    <t>DEF-007, DEF-008</t>
+    <t/>
   </si>
   <si>
     <t>resolved</t>
-  </si>
-  <si>
-    <t>DEF-004, DEF-005, DEF-006, DEF-009</t>
   </si>
 </sst>
 </file>
@@ -759,7 +753,7 @@
         <v>62</v>
       </c>
       <c r="C3" s="2">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -770,7 +764,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -781,7 +775,7 @@
         <v>95.4</v>
       </c>
       <c r="C5" s="2">
-        <v>95.2</v>
+        <v>98.8</v>
       </c>
     </row>
   </sheetData>
@@ -828,23 +822,23 @@
         <v>40</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
agentic-qe-mvp: execution hand-over delivers the evidence the EQE skill requires
Co-Authored-By: Devin AI <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/agentic-qe-mvp/demo-artifacts/comparison/compare-CYC-2-vs-CYC-3.xlsx
+++ b/agentic-qe-mvp/demo-artifacts/comparison/compare-CYC-2-vs-CYC-3.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="43">
   <si>
     <t>Artifact</t>
   </si>
@@ -133,16 +133,13 @@
     <t>CYC-3 defects</t>
   </si>
   <si>
-    <t>DEF-010</t>
+    <t/>
   </si>
   <si>
     <t>new</t>
   </si>
   <si>
     <t>still open</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>resolved</t>
@@ -753,7 +750,7 @@
         <v>62</v>
       </c>
       <c r="C3" s="2">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -764,7 +761,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -775,7 +772,7 @@
         <v>95.4</v>
       </c>
       <c r="C5" s="2">
-        <v>98.8</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -830,12 +827,12 @@
         <v>41</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>37</v>

</xml_diff>